<commit_message>
Manual: capturas de administración, informe e instalación en un ordenador
</commit_message>
<xml_diff>
--- a/datos/bibliotecas.xlsx
+++ b/datos/bibliotecas.xlsx
@@ -202,11 +202,6 @@
         <t>Superficie útil en metros cuadrados. Columna OPCIONAL: si se deja vacía, el indicador de documentos por m² aparece como «N/D».</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Clave de acceso, OPCIONAL. Con ella la biblioteca entra a su último análisis guardado sin subir los ficheros: escribe el nombre de la biblioteca y esta clave. La pone y la cambia el administrador de la red. Vacía = sin acceso con clave. No compartas este fichero con las claves puestas.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -507,7 +502,6 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -532,11 +526,6 @@
           <t>Metros_cuadrados</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Clave</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -553,7 +542,6 @@
       <c r="D2" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="E2" s="2" t="n"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Borra las tres filas de ejemplo y escribe debajo tus bibliotecas, una por fila.</t>
@@ -575,7 +563,6 @@
       <c r="D3" s="2" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="2" t="n"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>No cambies los nombres de la primera fila.</t>
@@ -595,12 +582,6 @@
         <v>628</v>
       </c>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>La columna Clave es opcional: ver su comentario.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -614,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -683,65 +664,58 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Clave               Opcional. Clave para entrar al último análisis guardado sin subir ficheros.</t>
-        </is>
-      </c>
+      <c r="A11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr"/>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Cómo saber el código de sucursal</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Cómo saber el código de sucursal</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Abre cualquier listado topográfico exportado de AbsysNet: la columna «Suc.» trae</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Abre cualquier listado topográfico exportado de AbsysNet: la columna «Suc.» trae</t>
+          <t>ese número en todas las líneas. Es el mismo para toda la biblioteca.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>ese número en todas las líneas. Es el mismo para toda la biblioteca.</t>
-        </is>
-      </c>
+      <c r="A15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Si no usas Excel</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Si no usas Excel</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Puedes guardar el mismo contenido como datos/bibliotecas.csv, con las mismas</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Puedes guardar el mismo contenido como datos/bibliotecas.csv, con las mismas</t>
+          <t>cuatro columnas en la primera fila. Bildumargi lo lee igual.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>columnas en la primera fila. Bildumargi lo lee igual.</t>
-        </is>
-      </c>
+      <c r="A19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Created by: Asier Urkia. Contact: bildumargi@gmail.com</t>
         </is>

</xml_diff>